<commit_message>
Some modification regading stopping criteria results. The modified results are used in the paper before sent it to co-authors
</commit_message>
<xml_diff>
--- a/SC reuslts/some results SPEA2.xlsx
+++ b/SC reuslts/some results SPEA2.xlsx
@@ -1,15 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahbub\Documents\GitHub\EnergyPLANDomainKnowledgeEAStep1\SC reuslts\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11385" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="11385" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="ZDT1" sheetId="1" r:id="rId1"/>
@@ -18,11 +13,12 @@
     <sheet name="ZDT4" sheetId="4" r:id="rId4"/>
     <sheet name="ZDT6" sheetId="5" r:id="rId5"/>
     <sheet name="DTLZ2" sheetId="6" r:id="rId6"/>
+    <sheet name="DTLZ5" sheetId="8" r:id="rId7"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="10">
   <si>
     <t>terminate generation</t>
   </si>
@@ -67,8 +63,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,17 +142,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:date1904 val="0"/>
   <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
@@ -189,8 +175,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
-      <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -198,33 +182,11 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="it-IT"/>
-        </a:p>
-      </c:txPr>
     </c:title>
-    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
         <c:scatterStyle val="smoothMarker"/>
-        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -1748,23 +1710,14 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="355980544"/>
-        <c:axId val="355979760"/>
+        <c:axId val="43150336"/>
+        <c:axId val="43177088"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="355980544"/>
+        <c:axId val="43150336"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:majorGridlines>
           <c:spPr>
@@ -1806,8 +1759,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
-          <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -1815,29 +1766,8 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="it-IT"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -1869,19 +1799,18 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="it-IT"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="355979760"/>
+        <c:crossAx val="43177088"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="355979760"/>
+        <c:axId val="43177088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
@@ -1923,8 +1852,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
-          <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -1932,30 +1859,9 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="it-IT"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -1987,10 +1893,10 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="it-IT"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="355980544"/>
+        <c:crossAx val="43150336"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2004,7 +1910,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2028,571 +1933,15 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="it-IT"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageMargins b="0.75000000000000022" l="0.70000000000000018" r="0.70000000000000018" t="0.75000000000000022" header="0.3000000000000001" footer="0.3000000000000001"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3201,7 +2550,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Sheet1"/>
@@ -5754,7 +5103,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -5789,7 +5138,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -5966,16 +5315,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
@@ -5985,7 +5334,7 @@
     <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -5999,7 +5348,7 @@
         <v>0.66616012487499998</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -6019,7 +5368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" s="4">
         <v>0</v>
       </c>
@@ -6039,7 +5388,7 @@
         <v>-4.02775403213009E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" s="4">
         <v>1</v>
       </c>
@@ -6059,7 +5408,7 @@
         <v>3.1351622381991999E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" s="4">
         <v>2</v>
       </c>
@@ -6079,7 +5428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7" s="4">
         <v>3</v>
       </c>
@@ -6099,7 +5448,7 @@
         <v>3.5947162432393501E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8" s="4">
         <v>4</v>
       </c>
@@ -6119,7 +5468,7 @@
         <v>2.8522046475236702E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9" s="4">
         <v>5</v>
       </c>
@@ -6139,7 +5488,7 @@
         <v>3.6982122083177799E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10" s="4">
         <v>6</v>
       </c>
@@ -6159,7 +5508,7 @@
         <v>-2.7118335422688599E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>7</v>
       </c>
@@ -6179,7 +5528,7 @@
         <v>-1.2344848441289101E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>8</v>
       </c>
@@ -6199,7 +5548,7 @@
         <v>-6.4374001771883005E-4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>9</v>
       </c>
@@ -6219,7 +5568,7 @@
         <v>6.2472665566742902E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>10</v>
       </c>
@@ -6239,7 +5588,7 @@
         <v>1.2462163371180701E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>11</v>
       </c>
@@ -6259,7 +5608,7 @@
         <v>3.2980982086585598E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>12</v>
       </c>
@@ -6279,7 +5628,7 @@
         <v>1.5353722018479701E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>13</v>
       </c>
@@ -6299,7 +5648,7 @@
         <v>-1.52577647807916E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>14</v>
       </c>
@@ -6319,7 +5668,7 @@
         <v>-6.3733362332385403E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>15</v>
       </c>
@@ -6339,7 +5688,7 @@
         <v>2.8183815968217899E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>16</v>
       </c>
@@ -6359,7 +5708,7 @@
         <v>1.6771180654425999E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>17</v>
       </c>
@@ -6379,7 +5728,7 @@
         <v>2.1832283042739699E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>18</v>
       </c>
@@ -6399,7 +5748,7 @@
         <v>-8.9656101168417103E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>19</v>
       </c>
@@ -6419,7 +5768,7 @@
         <v>3.0776962678815399E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>20</v>
       </c>
@@ -6439,7 +5788,7 @@
         <v>3.0787657958864499E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>21</v>
       </c>
@@ -6459,7 +5808,7 @@
         <v>-4.6952727690963703E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>22</v>
       </c>
@@ -6479,7 +5828,7 @@
         <v>3.5105583022494199E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>23</v>
       </c>
@@ -6499,7 +5848,7 @@
         <v>1.94843331581862E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>24</v>
       </c>
@@ -6519,7 +5868,7 @@
         <v>2.54959487698086E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>25</v>
       </c>
@@ -6539,7 +5888,7 @@
         <v>3.1356004368674399E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>26</v>
       </c>
@@ -6559,7 +5908,7 @@
         <v>5.0453275062578497E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>27</v>
       </c>
@@ -6579,7 +5928,7 @@
         <v>2.18397480503174E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>28</v>
       </c>
@@ -6599,7 +5948,7 @@
         <v>-3.6582652465511002E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6">
       <c r="A33">
         <v>29</v>
       </c>
@@ -6619,7 +5968,7 @@
         <v>-8.77236162429073E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -6643,9 +5992,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -6655,7 +6004,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -6669,7 +6018,7 @@
         <v>0.33283355941638099</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -6689,7 +6038,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>0</v>
       </c>
@@ -6709,7 +6058,7 @@
         <v>3.8523055154125602E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>1</v>
       </c>
@@ -6729,7 +6078,7 @@
         <v>8.9255436327625205E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>2</v>
       </c>
@@ -6749,7 +6098,7 @@
         <v>1.2864690327620801E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>3</v>
       </c>
@@ -6769,7 +6118,7 @@
         <v>3.5789596609926899E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>4</v>
       </c>
@@ -6789,7 +6138,7 @@
         <v>2.86906274243881E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>5</v>
       </c>
@@ -6809,7 +6158,7 @@
         <v>1.8742756194701799E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>6</v>
       </c>
@@ -6829,7 +6178,7 @@
         <v>7.5921083603877797E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>7</v>
       </c>
@@ -6849,7 +6198,7 @@
         <v>2.8288248501487602E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>8</v>
       </c>
@@ -6869,7 +6218,7 @@
         <v>2.0039067560449998E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>9</v>
       </c>
@@ -6889,7 +6238,7 @@
         <v>1.802300296295E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>10</v>
       </c>
@@ -6909,7 +6258,7 @@
         <v>0.50826848387610402</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>11</v>
       </c>
@@ -6929,7 +6278,7 @@
         <v>4.5363711615490302E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>12</v>
       </c>
@@ -6949,7 +6298,7 @@
         <v>1.05064870934321E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>13</v>
       </c>
@@ -6969,7 +6318,7 @@
         <v>1.0440257767501101E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>14</v>
       </c>
@@ -6989,7 +6338,7 @@
         <v>0.274448081519169</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>15</v>
       </c>
@@ -7009,7 +6358,7 @@
         <v>0.38361754664286202</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>16</v>
       </c>
@@ -7029,7 +6378,7 @@
         <v>-1.0786007040664001E-4</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>17</v>
       </c>
@@ -7049,7 +6398,7 @@
         <v>3.04817507616511E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>18</v>
       </c>
@@ -7069,7 +6418,7 @@
         <v>4.1940976844343503E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>19</v>
       </c>
@@ -7089,7 +6438,7 @@
         <v>7.1211896071660097E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>20</v>
       </c>
@@ -7109,7 +6458,7 @@
         <v>6.6526545502562798E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>21</v>
       </c>
@@ -7129,7 +6478,7 @@
         <v>5.1954422990063698E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>22</v>
       </c>
@@ -7149,7 +6498,7 @@
         <v>1.81615678061086E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>23</v>
       </c>
@@ -7169,7 +6518,7 @@
         <v>-5.6107163235391501E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>24</v>
       </c>
@@ -7189,7 +6538,7 @@
         <v>4.78926633556022E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>25</v>
       </c>
@@ -7209,7 +6558,7 @@
         <v>2.8284088861917299E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>26</v>
       </c>
@@ -7229,7 +6578,7 @@
         <v>3.7980373392806901E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>27</v>
       </c>
@@ -7249,7 +6598,7 @@
         <v>8.1718573538280804E-4</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>28</v>
       </c>
@@ -7269,7 +6618,7 @@
         <v>3.2910026702049301E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7">
       <c r="A33">
         <v>29</v>
       </c>
@@ -7289,7 +6638,7 @@
         <v>5.6122652139269204E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -7305,7 +6654,7 @@
         <v>0.98119115751499442</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7">
       <c r="D39">
         <f>QUARTILE($D$4:$D$33,0)</f>
         <v>-7.3447463576227806E-2</v>
@@ -7319,7 +6668,7 @@
         <v>-5.6107163235391501E-4</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7">
       <c r="D40">
         <f>QUARTILE($D$4:$D$33,1)</f>
         <v>-5.3929254327688128E-3</v>
@@ -7333,7 +6682,7 @@
         <v>1.0489929761949351E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7">
       <c r="D41">
         <f>QUARTILE($D$4:$D$33,2)</f>
         <v>-3.3406997323205349E-3</v>
@@ -7347,7 +6696,7 @@
         <v>2.8489437962937849E-3</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7">
       <c r="D42">
         <f>QUARTILE($D$4:$D$33,3)</f>
         <v>-2.2995423403989975E-3</v>
@@ -7361,7 +6710,7 @@
         <v>4.805344674643503E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7">
       <c r="D43">
         <f>QUARTILE($D$4:$D$33,4)</f>
         <v>-2.9951742651201902E-4</v>
@@ -7375,7 +6724,7 @@
         <v>0.50826848387610402</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7">
       <c r="D45">
         <f>D38-D37</f>
         <v>0</v>
@@ -7385,7 +6734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7">
       <c r="D46">
         <f>D39-D38</f>
         <v>-7.3447463576227806E-2</v>
@@ -7395,7 +6744,7 @@
         <v>5.6107163235391501E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7">
       <c r="D47">
         <f t="shared" ref="D47:D50" si="0">D40-D39</f>
         <v>6.8054538143458992E-2</v>
@@ -7405,7 +6754,7 @@
         <v>-1.6100646085488502E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7">
       <c r="D48">
         <f t="shared" si="0"/>
         <v>2.0522257004482779E-3</v>
@@ -7415,7 +6764,7 @@
         <v>-1.7999508200988498E-3</v>
       </c>
     </row>
-    <row r="49" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:6">
       <c r="D49">
         <f t="shared" si="0"/>
         <v>1.0411573919215373E-3</v>
@@ -7425,7 +6774,7 @@
         <v>-1.9564008783497181E-3</v>
       </c>
     </row>
-    <row r="50" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="4:6">
       <c r="D50">
         <f t="shared" si="0"/>
         <v>2.0000249138869787E-3</v>
@@ -7442,9 +6791,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -7454,7 +6803,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -7468,7 +6817,7 @@
         <v>0.51719187154758695</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -7488,7 +6837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>0</v>
       </c>
@@ -7508,7 +6857,7 @@
         <v>-2.2807006902435499E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>1</v>
       </c>
@@ -7528,7 +6877,7 @@
         <v>1.8337801287048199E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>2</v>
       </c>
@@ -7548,7 +6897,7 @@
         <v>1.70843410751445E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>3</v>
       </c>
@@ -7568,7 +6917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>4</v>
       </c>
@@ -7588,7 +6937,7 @@
         <v>-1.9512732532300699E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>5</v>
       </c>
@@ -7608,7 +6957,7 @@
         <v>2.2421997582870098E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>6</v>
       </c>
@@ -7628,7 +6977,7 @@
         <v>2.7931703548921801E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>7</v>
       </c>
@@ -7648,7 +6997,7 @@
         <v>-3.9834054963709599E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>8</v>
       </c>
@@ -7668,7 +7017,7 @@
         <v>3.4601407434816898E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>9</v>
       </c>
@@ -7688,7 +7037,7 @@
         <v>9.0711773134788398E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>10</v>
       </c>
@@ -7708,7 +7057,7 @@
         <v>-7.5750863865021497E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>11</v>
       </c>
@@ -7728,7 +7077,7 @@
         <v>4.3150980055167397E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>12</v>
       </c>
@@ -7748,7 +7097,7 @@
         <v>1.12457626755606E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>13</v>
       </c>
@@ -7768,7 +7117,7 @@
         <v>-3.7266454008523702E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>14</v>
       </c>
@@ -7788,7 +7137,7 @@
         <v>2.0184466823093901E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>15</v>
       </c>
@@ -7808,7 +7157,7 @@
         <v>-2.9035944088125001E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>16</v>
       </c>
@@ -7828,7 +7177,7 @@
         <v>-5.8757895288296998E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>17</v>
       </c>
@@ -7848,7 +7197,7 @@
         <v>5.8036199420665102E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>18</v>
       </c>
@@ -7868,7 +7217,7 @@
         <v>-1.21371351810894E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>19</v>
       </c>
@@ -7888,7 +7237,7 @@
         <v>1.0280245421169E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>20</v>
       </c>
@@ -7908,7 +7257,7 @@
         <v>2.3265224199887002E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>21</v>
       </c>
@@ -7928,7 +7277,7 @@
         <v>-5.3253045064557102E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>22</v>
       </c>
@@ -7948,7 +7297,7 @@
         <v>-0.13072853269083401</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>23</v>
       </c>
@@ -7968,7 +7317,7 @@
         <v>1.1887513924489701E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>24</v>
       </c>
@@ -7988,7 +7337,7 @@
         <v>-4.8468769372609901E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>25</v>
       </c>
@@ -8008,7 +7357,7 @@
         <v>6.1630899999999501E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>26</v>
       </c>
@@ -8028,7 +7377,7 @@
         <v>-1.44404672564077E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>27</v>
       </c>
@@ -8048,7 +7397,7 @@
         <v>-2.7000402398105099E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>28</v>
       </c>
@@ -8068,7 +7417,7 @@
         <v>2.4655135084373698E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6">
       <c r="A33">
         <v>29</v>
       </c>
@@ -8088,7 +7437,7 @@
         <v>3.9909273234590903E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -8104,7 +7453,7 @@
         <v>0.98531081408259802</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6">
       <c r="D39">
         <f>QUARTILE($D$4:$D$33,0)</f>
         <v>-4.8503293867775401E-3</v>
@@ -8114,7 +7463,7 @@
         <v>-0.13072853269083401</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6">
       <c r="D40">
         <f>QUARTILE($D$4:$D$33,1)</f>
         <v>-2.3685920106444026E-3</v>
@@ -8124,7 +7473,7 @@
         <v>-2.5952053524187701E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6">
       <c r="D41">
         <f>QUARTILE($D$4:$D$33,2)</f>
         <v>8.6634067526402748E-5</v>
@@ -8134,7 +7483,7 @@
         <v>7.617133656739395E-4</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6">
       <c r="D42">
         <f>QUARTILE($D$4:$D$33,3)</f>
         <v>1.3713860752048975E-3</v>
@@ -8144,7 +7493,7 @@
         <v>2.1862614892926048E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6">
       <c r="D43">
         <f>QUARTILE($D$4:$D$33,4)</f>
         <v>7.7068485576757897E-2</v>
@@ -8154,7 +7503,7 @@
         <v>5.8036199420665102E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6">
       <c r="D45">
         <f>D38-D37</f>
         <v>0</v>
@@ -8164,7 +7513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6">
       <c r="D46">
         <f>D39-D38</f>
         <v>-4.8503293867775401E-3</v>
@@ -8174,7 +7523,7 @@
         <v>-0.13072853269083401</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6">
       <c r="D47">
         <f t="shared" ref="D47:F50" si="0">D40-D39</f>
         <v>2.4817373761331376E-3</v>
@@ -8184,7 +7533,7 @@
         <v>0.12813332733841523</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6">
       <c r="D48">
         <f t="shared" si="0"/>
         <v>2.4552260781708054E-3</v>
@@ -8194,7 +7543,7 @@
         <v>3.3569187180927098E-3</v>
       </c>
     </row>
-    <row r="49" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:6">
       <c r="D49">
         <f t="shared" si="0"/>
         <v>1.2847520076784947E-3</v>
@@ -8204,7 +7553,7 @@
         <v>1.4245481236186653E-3</v>
       </c>
     </row>
-    <row r="50" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="4:6">
       <c r="D50">
         <f t="shared" si="0"/>
         <v>7.5697099501552997E-2</v>
@@ -8221,9 +7570,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -8233,7 +7582,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -8247,7 +7596,7 @@
         <v>0.66617361728492197</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -8267,7 +7616,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>0</v>
       </c>
@@ -8287,7 +7636,7 @@
         <v>0.12641769222756899</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>1</v>
       </c>
@@ -8307,7 +7656,7 @@
         <v>0.23609067374838499</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>2</v>
       </c>
@@ -8327,7 +7676,7 @@
         <v>-0.27580101308231197</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>3</v>
       </c>
@@ -8347,7 +7696,7 @@
         <v>-0.399486082564184</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>4</v>
       </c>
@@ -8367,7 +7716,7 @@
         <v>0.24845030235641</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>5</v>
       </c>
@@ -8387,7 +7736,7 @@
         <v>0.18877196182539999</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>6</v>
       </c>
@@ -8407,7 +7756,7 @@
         <v>7.9895529873842699E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>7</v>
       </c>
@@ -8427,7 +7776,7 @@
         <v>7.0897684882383197E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>8</v>
       </c>
@@ -8447,7 +7796,7 @@
         <v>-0.30976012065077302</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>9</v>
       </c>
@@ -8467,7 +7816,7 @@
         <v>6.6116976577093303E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>10</v>
       </c>
@@ -8487,7 +7836,7 @@
         <v>0.180635135401638</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>11</v>
       </c>
@@ -8507,7 +7856,7 @@
         <v>4.44655507247637E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>12</v>
       </c>
@@ -8527,7 +7876,7 @@
         <v>0.261077185217644</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>13</v>
       </c>
@@ -8547,7 +7896,7 @@
         <v>0.16608733095460099</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>14</v>
       </c>
@@ -8567,7 +7916,7 @@
         <v>-1.239270585741</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>15</v>
       </c>
@@ -8587,7 +7936,7 @@
         <v>0.240466646099638</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>16</v>
       </c>
@@ -8607,7 +7956,7 @@
         <v>6.4365504239146498E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>17</v>
       </c>
@@ -8627,7 +7976,7 @@
         <v>0.28987547304325401</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>18</v>
       </c>
@@ -8647,7 +7996,7 @@
         <v>0.26564846897187799</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>19</v>
       </c>
@@ -8667,7 +8016,7 @@
         <v>0.16570935656639399</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>20</v>
       </c>
@@ -8687,7 +8036,7 @@
         <v>0.144188608602076</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>21</v>
       </c>
@@ -8707,7 +8056,7 @@
         <v>0.18894053716050599</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>22</v>
       </c>
@@ -8727,7 +8076,7 @@
         <v>0.247010951439184</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>23</v>
       </c>
@@ -8747,7 +8096,7 @@
         <v>2.5186997760617402E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>24</v>
       </c>
@@ -8767,7 +8116,7 @@
         <v>7.2015658468263299E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>25</v>
       </c>
@@ -8787,7 +8136,7 @@
         <v>0.279743046920302</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>26</v>
       </c>
@@ -8807,7 +8156,7 @@
         <v>0.16603459692549499</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>27</v>
       </c>
@@ -8827,7 +8176,7 @@
         <v>9.9101011393004593E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>28</v>
       </c>
@@ -8847,7 +8196,7 @@
         <v>1.23126229692725E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6">
       <c r="A33">
         <v>29</v>
       </c>
@@ -8867,7 +8216,7 @@
         <v>0.27668192501396599</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -8889,9 +8238,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -8901,7 +8250,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -8915,7 +8264,7 @@
         <v>0.40590724234006298</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -8935,7 +8284,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>0</v>
       </c>
@@ -8955,7 +8304,7 @@
         <v>5.0445725142826497E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>1</v>
       </c>
@@ -8975,7 +8324,7 @@
         <v>4.8536956978391901E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>2</v>
       </c>
@@ -8995,7 +8344,7 @@
         <v>6.6177501914829906E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>3</v>
       </c>
@@ -9015,7 +8364,7 @@
         <v>6.6082616067823896E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>4</v>
       </c>
@@ -9035,7 +8384,7 @@
         <v>-0.75205895691092395</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>5</v>
       </c>
@@ -9055,7 +8404,7 @@
         <v>-1.8171025605656099</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>6</v>
       </c>
@@ -9075,7 +8424,7 @@
         <v>4.9336616955308402E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>7</v>
       </c>
@@ -9095,7 +8444,7 @@
         <v>-1.0579869865467799</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>8</v>
       </c>
@@ -9115,7 +8464,7 @@
         <v>6.21121860082492E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>9</v>
       </c>
@@ -9135,7 +8484,7 @@
         <v>-0.79446630271998997</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>10</v>
       </c>
@@ -9155,7 +8504,7 @@
         <v>5.1458381567419297E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>11</v>
       </c>
@@ -9175,7 +8524,7 @@
         <v>4.2373727246239598E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>12</v>
       </c>
@@ -9195,7 +8544,7 @@
         <v>4.9940598405089201E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>13</v>
       </c>
@@ -9215,7 +8564,7 @@
         <v>4.3822562973532597E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>14</v>
       </c>
@@ -9235,7 +8584,7 @@
         <v>5.8738885450615202E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>15</v>
       </c>
@@ -9255,7 +8604,7 @@
         <v>3.5848818266332197E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>16</v>
       </c>
@@ -9275,7 +8624,7 @@
         <v>-0.74558394147236795</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>17</v>
       </c>
@@ -9295,7 +8644,7 @@
         <v>5.7637636293753097E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>18</v>
       </c>
@@ -9315,7 +8664,7 @@
         <v>3.85787779620098E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>19</v>
       </c>
@@ -9335,7 +8684,7 @@
         <v>5.0764843379359E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>20</v>
       </c>
@@ -9355,7 +8704,7 @@
         <v>5.0366316355794798E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>21</v>
       </c>
@@ -9375,7 +8724,7 @@
         <v>4.1224855188961698E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>22</v>
       </c>
@@ -9395,7 +8744,7 @@
         <v>4.6482406096914002E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>23</v>
       </c>
@@ -9415,7 +8764,7 @@
         <v>4.3003504241371698E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>24</v>
       </c>
@@ -9435,7 +8784,7 @@
         <v>3.7041761377940498E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>25</v>
       </c>
@@ -9455,7 +8804,7 @@
         <v>6.8682376237622397E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>26</v>
       </c>
@@ -9475,7 +8824,7 @@
         <v>7.3528199136519395E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>27</v>
       </c>
@@ -9495,7 +8844,7 @@
         <v>-0.502950940179553</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>28</v>
       </c>
@@ -9515,7 +8864,7 @@
         <v>3.9898329048502199E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6">
       <c r="A33">
         <v>29</v>
       </c>
@@ -9535,7 +8884,7 @@
         <v>5.6495673803255701E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -9551,7 +8900,7 @@
         <v>0.78901180554458616</v>
       </c>
     </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="6:6">
       <c r="F55" s="1"/>
     </row>
   </sheetData>
@@ -9566,9 +8915,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -9578,7 +8927,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -9592,7 +8941,7 @@
         <v>0.46783583650461702</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -9612,7 +8961,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>0</v>
       </c>
@@ -9632,7 +8981,7 @@
         <v>2.41894361971228E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>1</v>
       </c>
@@ -9652,7 +9001,7 @@
         <v>9.4184950611304608E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>2</v>
       </c>
@@ -9672,7 +9021,7 @@
         <v>7.4072554880356602E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>3</v>
       </c>
@@ -9692,7 +9041,7 @@
         <v>9.6830525324004199E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>4</v>
       </c>
@@ -9712,7 +9061,7 @@
         <v>-6.2258725178009301E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>5</v>
       </c>
@@ -9732,7 +9081,7 @@
         <v>1.0912163952796899E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>6</v>
       </c>
@@ -9752,7 +9101,7 @@
         <v>-1.1476083954315999E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>7</v>
       </c>
@@ -9772,7 +9121,7 @@
         <v>-2.7941881277670701E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>8</v>
       </c>
@@ -9792,7 +9141,7 @@
         <v>1.28330925438553E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>9</v>
       </c>
@@ -9812,7 +9161,7 @@
         <v>1.6348332850218101E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>10</v>
       </c>
@@ -9832,7 +9181,7 @@
         <v>3.7285562679005798E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>11</v>
       </c>
@@ -9852,7 +9201,7 @@
         <v>6.4685116879062898E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>12</v>
       </c>
@@ -9872,7 +9221,7 @@
         <v>-1.78977973209437E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>13</v>
       </c>
@@ -9892,7 +9241,7 @@
         <v>-1.37761608985909E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>14</v>
       </c>
@@ -9912,7 +9261,7 @@
         <v>-1.21767550640211E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>15</v>
       </c>
@@ -9932,7 +9281,7 @@
         <v>-2.0207482958943802E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>16</v>
       </c>
@@ -9952,7 +9301,7 @@
         <v>-6.11859052617087E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>17</v>
       </c>
@@ -9972,7 +9321,7 @@
         <v>4.13129728437366E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>18</v>
       </c>
@@ -9992,7 +9341,7 @@
         <v>1.11314132588568E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>19</v>
       </c>
@@ -10012,7 +9361,7 @@
         <v>2.2537277481197299E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>20</v>
       </c>
@@ -10032,7 +9381,7 @@
         <v>1.6605586224087399E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>21</v>
       </c>
@@ -10052,7 +9401,7 @@
         <v>-2.20356715835778E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>22</v>
       </c>
@@ -10072,7 +9421,7 @@
         <v>-6.1286501968491596E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>23</v>
       </c>
@@ -10092,7 +9441,7 @@
         <v>-2.04225772857256E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>24</v>
       </c>
@@ -10112,7 +9461,7 @@
         <v>-4.5254116492518398E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>25</v>
       </c>
@@ -10132,7 +9481,7 @@
         <v>-8.6370126225220299E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>26</v>
       </c>
@@ -10152,7 +9501,7 @@
         <v>1.0620176477237301E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>27</v>
       </c>
@@ -10172,7 +9521,7 @@
         <v>9.0254622444018301E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>28</v>
       </c>
@@ -10192,7 +9541,7 @@
         <v>-1.76621808816891E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6">
       <c r="A33">
         <v>29</v>
       </c>
@@ -10212,7 +9561,7 @@
         <v>-1.37904708023407E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -10226,6 +9575,674 @@
       <c r="E34">
         <f>AVERAGE(E4:E33)</f>
         <v>0.85751866938468002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1">
+        <v>200</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1">
+        <v>9.5583254269994297E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>89</v>
+      </c>
+      <c r="C4">
+        <v>11100</v>
+      </c>
+      <c r="D4">
+        <v>2.10658847006324E-3</v>
+      </c>
+      <c r="E4">
+        <v>0.94684976264012199</v>
+      </c>
+      <c r="F4">
+        <v>-5.2242760335330296E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>419</v>
+      </c>
+      <c r="C5">
+        <v>-21900</v>
+      </c>
+      <c r="D5" s="1">
+        <v>-5.8684472604744698E-4</v>
+      </c>
+      <c r="E5">
+        <v>0.97631221369139298</v>
+      </c>
+      <c r="F5">
+        <v>1.0109118381800199E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>84</v>
+      </c>
+      <c r="C6">
+        <v>11600</v>
+      </c>
+      <c r="D6">
+        <v>2.0930265203309901E-3</v>
+      </c>
+      <c r="E6">
+        <v>0.95237250241049098</v>
+      </c>
+      <c r="F6">
+        <v>-1.95846461746285E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>77</v>
+      </c>
+      <c r="C7">
+        <v>12300</v>
+      </c>
+      <c r="D7" s="1">
+        <v>3.0809628333879702E-3</v>
+      </c>
+      <c r="E7">
+        <v>0.94431185566363396</v>
+      </c>
+      <c r="F7" s="1">
+        <v>-2.1328006759585498E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>76</v>
+      </c>
+      <c r="C8">
+        <v>12400</v>
+      </c>
+      <c r="D8" s="1">
+        <v>4.3594652387582899E-3</v>
+      </c>
+      <c r="E8">
+        <v>0.92737796477991397</v>
+      </c>
+      <c r="F8">
+        <v>-6.5108424817733003E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>88</v>
+      </c>
+      <c r="C9">
+        <v>11200</v>
+      </c>
+      <c r="D9">
+        <v>1.64544161179437E-3</v>
+      </c>
+      <c r="E9">
+        <v>0.95467302175826896</v>
+      </c>
+      <c r="F9">
+        <v>-3.42965240311388E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10">
+        <v>102</v>
+      </c>
+      <c r="C10">
+        <v>9800</v>
+      </c>
+      <c r="D10">
+        <v>1.70275215063259E-3</v>
+      </c>
+      <c r="E10">
+        <v>0.95838978149313603</v>
+      </c>
+      <c r="F10">
+        <v>-3.8742538803804801E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>107</v>
+      </c>
+      <c r="C11">
+        <v>9300</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1.40818298951674E-3</v>
+      </c>
+      <c r="E11">
+        <v>0.95833717634418003</v>
+      </c>
+      <c r="F11">
+        <v>-1.9166022357748301E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12">
+        <v>93</v>
+      </c>
+      <c r="C12">
+        <v>10700</v>
+      </c>
+      <c r="D12">
+        <v>1.90470563775468E-3</v>
+      </c>
+      <c r="E12">
+        <v>0.95181547376676501</v>
+      </c>
+      <c r="F12">
+        <v>-3.4359154587345602E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <v>88</v>
+      </c>
+      <c r="C13">
+        <v>11200</v>
+      </c>
+      <c r="D13">
+        <v>1.4244886890251399E-3</v>
+      </c>
+      <c r="E13">
+        <v>0.95877056342024103</v>
+      </c>
+      <c r="F13">
+        <v>-2.16589126147676E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14">
+        <v>130</v>
+      </c>
+      <c r="C14">
+        <v>7000</v>
+      </c>
+      <c r="D14" s="1">
+        <v>4.4538697104159997E-4</v>
+      </c>
+      <c r="E14">
+        <v>0.97035495982734299</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2.76360779528694E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15">
+        <v>11</v>
+      </c>
+      <c r="B15">
+        <v>344</v>
+      </c>
+      <c r="C15">
+        <v>-14400</v>
+      </c>
+      <c r="D15" s="1">
+        <v>-1.11601282585332E-4</v>
+      </c>
+      <c r="E15">
+        <v>0.97441072888179303</v>
+      </c>
+      <c r="F15" s="1">
+        <v>-7.4250580818913104E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16">
+        <v>12</v>
+      </c>
+      <c r="B16">
+        <v>236</v>
+      </c>
+      <c r="C16">
+        <v>-3600</v>
+      </c>
+      <c r="D16" s="1">
+        <v>-4.9144273220492996E-4</v>
+      </c>
+      <c r="E16">
+        <v>0.97657319814629195</v>
+      </c>
+      <c r="F16" s="1">
+        <v>2.2241594888672199E-4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17">
+        <v>13</v>
+      </c>
+      <c r="B17">
+        <v>123</v>
+      </c>
+      <c r="C17">
+        <v>7700</v>
+      </c>
+      <c r="D17" s="1">
+        <v>9.2596880348273704E-4</v>
+      </c>
+      <c r="E17">
+        <v>0.96544282738167597</v>
+      </c>
+      <c r="F17" s="1">
+        <v>-1.2316503781557499E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18">
+        <v>14</v>
+      </c>
+      <c r="B18">
+        <v>191</v>
+      </c>
+      <c r="C18">
+        <v>900</v>
+      </c>
+      <c r="D18" s="1">
+        <v>2.9509015628147102E-4</v>
+      </c>
+      <c r="E18">
+        <v>0.97125013148256001</v>
+      </c>
+      <c r="F18" s="1">
+        <v>-1.5274381637497801E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19">
+        <v>15</v>
+      </c>
+      <c r="B19">
+        <v>102</v>
+      </c>
+      <c r="C19">
+        <v>9800</v>
+      </c>
+      <c r="D19">
+        <v>1.30626921906651E-3</v>
+      </c>
+      <c r="E19">
+        <v>0.95841603660946195</v>
+      </c>
+      <c r="F19" s="1">
+        <v>-2.28178988861293E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20">
+        <v>16</v>
+      </c>
+      <c r="B20">
+        <v>125</v>
+      </c>
+      <c r="C20">
+        <v>7500</v>
+      </c>
+      <c r="D20" s="1">
+        <v>6.3425879394915497E-4</v>
+      </c>
+      <c r="E20">
+        <v>0.96630710902040395</v>
+      </c>
+      <c r="F20" s="1">
+        <v>-9.8763005355828604E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21">
+        <v>17</v>
+      </c>
+      <c r="B21">
+        <v>194</v>
+      </c>
+      <c r="C21">
+        <v>600</v>
+      </c>
+      <c r="D21" s="1">
+        <v>1.6297981431992399E-4</v>
+      </c>
+      <c r="E21">
+        <v>0.96838992739061402</v>
+      </c>
+      <c r="F21" s="1">
+        <v>3.8852833327827001E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22">
+        <v>18</v>
+      </c>
+      <c r="B22">
+        <v>102</v>
+      </c>
+      <c r="C22">
+        <v>9800</v>
+      </c>
+      <c r="D22" s="1">
+        <v>7.5451235957445196E-4</v>
+      </c>
+      <c r="E22">
+        <v>0.96459018710254696</v>
+      </c>
+      <c r="F22" s="1">
+        <v>-1.22004643815976E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23">
+        <v>19</v>
+      </c>
+      <c r="B23">
+        <v>192</v>
+      </c>
+      <c r="C23">
+        <v>800</v>
+      </c>
+      <c r="D23" s="1">
+        <v>1.12959564144601E-4</v>
+      </c>
+      <c r="E23">
+        <v>0.97419068795572605</v>
+      </c>
+      <c r="F23" s="1">
+        <v>-8.5216287226152999E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24">
+        <v>20</v>
+      </c>
+      <c r="B24">
+        <v>118</v>
+      </c>
+      <c r="C24">
+        <v>8200</v>
+      </c>
+      <c r="D24" s="1">
+        <v>1.22780953872404E-3</v>
+      </c>
+      <c r="E24">
+        <v>0.96201129939014096</v>
+      </c>
+      <c r="F24">
+        <v>-2.06096371513386E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25">
+        <v>21</v>
+      </c>
+      <c r="B25">
+        <v>206</v>
+      </c>
+      <c r="C25">
+        <v>-600</v>
+      </c>
+      <c r="D25" s="1">
+        <v>-2.8622446976743401E-4</v>
+      </c>
+      <c r="E25">
+        <v>0.97362628624103797</v>
+      </c>
+      <c r="F25">
+        <v>1.17100064228736E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26">
+        <v>22</v>
+      </c>
+      <c r="B26">
+        <v>196</v>
+      </c>
+      <c r="C26">
+        <v>400</v>
+      </c>
+      <c r="D26" s="1">
+        <v>1.10018913124398E-4</v>
+      </c>
+      <c r="E26">
+        <v>0.97038476035681498</v>
+      </c>
+      <c r="F26">
+        <v>-1.1917659954188101E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27">
+        <v>23</v>
+      </c>
+      <c r="B27">
+        <v>117</v>
+      </c>
+      <c r="C27">
+        <v>8300</v>
+      </c>
+      <c r="D27" s="1">
+        <v>9.4764022362116198E-4</v>
+      </c>
+      <c r="E27">
+        <v>0.96445304239985896</v>
+      </c>
+      <c r="F27">
+        <v>1.4803297169123E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28">
+        <v>24</v>
+      </c>
+      <c r="B28">
+        <v>75</v>
+      </c>
+      <c r="C28">
+        <v>12500</v>
+      </c>
+      <c r="D28" s="1">
+        <v>3.5562730782175401E-3</v>
+      </c>
+      <c r="E28">
+        <v>0.93279823229676195</v>
+      </c>
+      <c r="F28" s="1">
+        <v>-4.0789013558030201E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29">
+        <v>25</v>
+      </c>
+      <c r="B29">
+        <v>90</v>
+      </c>
+      <c r="C29">
+        <v>11000</v>
+      </c>
+      <c r="D29" s="1">
+        <v>1.32764202108005E-3</v>
+      </c>
+      <c r="E29">
+        <v>0.95731814513258096</v>
+      </c>
+      <c r="F29" s="1">
+        <v>-4.4142500700672301E-4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30">
+        <v>26</v>
+      </c>
+      <c r="B30">
+        <v>150</v>
+      </c>
+      <c r="C30">
+        <v>5000</v>
+      </c>
+      <c r="D30" s="1">
+        <v>3.7488475641708698E-4</v>
+      </c>
+      <c r="E30">
+        <v>0.97345082656368598</v>
+      </c>
+      <c r="F30" s="1">
+        <v>-1.2113950797222801E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31">
+        <v>27</v>
+      </c>
+      <c r="B31">
+        <v>76</v>
+      </c>
+      <c r="C31">
+        <v>12400</v>
+      </c>
+      <c r="D31">
+        <v>2.62787815931371E-3</v>
+      </c>
+      <c r="E31">
+        <v>0.94702258438312104</v>
+      </c>
+      <c r="F31">
+        <v>-2.2650228081930101E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32">
+        <v>28</v>
+      </c>
+      <c r="B32">
+        <v>86</v>
+      </c>
+      <c r="C32">
+        <v>11400</v>
+      </c>
+      <c r="D32" s="1">
+        <v>1.75773465396693E-3</v>
+      </c>
+      <c r="E32">
+        <v>0.95539827117188703</v>
+      </c>
+      <c r="F32" s="1">
+        <v>9.65543453944617E-5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33">
+        <v>29</v>
+      </c>
+      <c r="B33">
+        <v>262</v>
+      </c>
+      <c r="C33">
+        <v>-6200</v>
+      </c>
+      <c r="D33" s="1">
+        <v>1.87343264214642E-4</v>
+      </c>
+      <c r="E33">
+        <v>0.97212790422658701</v>
+      </c>
+      <c r="F33" s="1">
+        <v>6.8535011062809104E-4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34">
+        <f>SUM(C4:C33)</f>
+        <v>166200</v>
+      </c>
+      <c r="D34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <f>AVERAGE(E4:E33)</f>
+        <v>0.96092424873096804</v>
       </c>
     </row>
   </sheetData>

</xml_diff>